<commit_message>
wgeel is so fun
</commit_message>
<xml_diff>
--- a/R/advice/advice_basis.xlsx
+++ b/R/advice/advice_basis.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuille1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Feuille1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -37,8 +37,8 @@
 HELCOM’s Baltic Sea Action Plan (BSAP) contains several targets for European eel [@helcom2021a].  
 National conservation measures are contained in the report of the Workshop for the Technical evaluation of EU Member States' Progress Reports for submission in 2022 and 2025 [@ices2022c; @ices2025], Eel Management Plan progress reports submitted in 2024, and the country reports of the Joint ICES/European Inland Fisheries and Aquaculture Advisory Commission (EIFAAC)/General Fisheries Commission for the Mediterranean (GFCM) Working Group on Eels [@ices2022a; @ices2024a]. 
 Other international legislations/communications relevant to eel conservation:  
-\- Directive 2000/60/EC, known as the Water Framework Directive (WFD; [@eu2000]) 
-\- Directive 2008/56/EC, known as the Marine Strategy Framework Directive (MSFD; [@eu2008]). 
+\- Directive 2000/60/EC, known as the Water Framework Directive [WFD - @eu2000] 
+\- Directive 2008/56/EC, known as the Marine Strategy Framework Directive [MSFD - @eu2008]. 
 \- Council Directive 92/43/EEC, known as the Habitats Directive [@eu1992] 
 \- The Ramsar Convention on Wetlands [@unitednations1976], which aims to stem the loss of and progressive encroachment on wetlands, an important European eel habitat.  
 \- EU Nature Restoration Law: Regulation (EU) 2024/1991 [@eu2024] 
@@ -118,16 +118,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -143,31 +147,137 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18A303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369A3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A33E03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8E03A3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="C99C00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="C9211E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000EE"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551A8B"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="37.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="80.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="37.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="80.03"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="394.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>